<commit_message>
docs: update technical documentation and data dictionary
</commit_message>
<xml_diff>
--- a/Diccionario_Datos_V2_Sincronizado.xlsx
+++ b/Diccionario_Datos_V2_Sincronizado.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12285"/>
+    <workbookView windowWidth="28800" windowHeight="12285" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="User" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="472" uniqueCount="137">
   <si>
     <t>Campo</t>
   </si>
@@ -321,6 +321,42 @@
   </si>
   <si>
     <t>Campo del Registro de Viajes y control de tickets (updatedAt).</t>
+  </si>
+  <si>
+    <t>cambio</t>
+  </si>
+  <si>
+    <t>add</t>
+  </si>
+  <si>
+    <t>6 Producto</t>
+  </si>
+  <si>
+    <t>ValorPorGalon</t>
+  </si>
+  <si>
+    <t>9 valor Flete</t>
+  </si>
+  <si>
+    <t>Valor Acpm</t>
+  </si>
+  <si>
+    <t>10 ACPM (Gal)</t>
+  </si>
+  <si>
+    <t>ValoeFerry</t>
+  </si>
+  <si>
+    <t>Destino</t>
+  </si>
+  <si>
+    <t>Empresa</t>
+  </si>
+  <si>
+    <t>ValorTonelada</t>
+  </si>
+  <si>
+    <t>PorcentajeConductor</t>
   </si>
   <si>
     <t>userId</t>
@@ -403,12 +439,12 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
-    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="42" formatCode="_-&quot;£&quot;* #,##0_-;\-&quot;£&quot;* #,##0_-;_-&quot;£&quot;* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -425,7 +461,21 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -435,13 +485,6 @@
       <color theme="0"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -462,21 +505,14 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="18"/>
+      <sz val="13"/>
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -485,7 +521,14 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -500,60 +543,14 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF3F3F3F"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
+      <sz val="18"/>
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -568,14 +565,59 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -584,7 +626,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -596,25 +638,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
+        <fgColor rgb="FFFFEB9C"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -632,7 +662,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -644,13 +686,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -662,19 +728,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -692,7 +758,31 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -704,67 +794,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5"/>
+        <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
+        <fgColor rgb="FFA5A5A5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
+        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -832,6 +880,41 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="double">
         <color rgb="FF3F3F3F"/>
       </left>
@@ -855,195 +938,166 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2988,7 +3042,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="14.1111111111111" customWidth="1"/>
@@ -3084,7 +3138,7 @@
       </c>
     </row>
     <row r="6" spans="1:5">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>57</v>
       </c>
       <c r="B6" s="2" t="s">
@@ -3101,19 +3155,19 @@
       </c>
     </row>
     <row r="7" spans="1:5">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" s="2" t="s">
+      <c r="C7" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" s="4" t="s">
         <v>70</v>
       </c>
     </row>
@@ -3135,7 +3189,7 @@
       </c>
     </row>
     <row r="9" spans="1:5">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>73</v>
       </c>
       <c r="B9" s="2" t="s">
@@ -3152,7 +3206,7 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>75</v>
       </c>
       <c r="B10" s="2" t="s">
@@ -3370,6 +3424,58 @@
       </c>
       <c r="E22" s="2" t="s">
         <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" t="s">
+        <v>100</v>
+      </c>
+      <c r="B24" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" t="s">
+        <v>102</v>
+      </c>
+      <c r="B25" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="B26" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="B27" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="28" spans="2:2">
+      <c r="B28" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="29" spans="2:2">
+      <c r="B29" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="30" spans="2:2">
+      <c r="B30" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="31" spans="2:2">
+      <c r="B31" t="s">
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -3430,7 +3536,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>6</v>
@@ -3442,12 +3548,12 @@
         <v>11</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>101</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="2" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>92</v>
@@ -3459,15 +3565,15 @@
         <v>35</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="2" t="s">
-        <v>104</v>
+        <v>116</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>7</v>
@@ -3476,12 +3582,12 @@
         <v>11</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>106</v>
+        <v>118</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="2" t="s">
-        <v>107</v>
+        <v>119</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>6</v>
@@ -3493,12 +3599,12 @@
         <v>11</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>108</v>
+        <v>120</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="2" t="s">
-        <v>109</v>
+        <v>121</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>6</v>
@@ -3510,15 +3616,15 @@
         <v>11</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="2" t="s">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>14</v>
@@ -3527,15 +3633,15 @@
         <v>11</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>113</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="2" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>112</v>
+        <v>124</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>14</v>
@@ -3544,12 +3650,12 @@
         <v>11</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>115</v>
+        <v>127</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="2" t="s">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>6</v>
@@ -3561,12 +3667,12 @@
         <v>11</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="2" t="s">
-        <v>118</v>
+        <v>130</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>6</v>
@@ -3578,7 +3684,7 @@
         <v>11</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -3595,7 +3701,7 @@
         <v>11</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
     </row>
   </sheetData>
@@ -3656,7 +3762,7 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>6</v>
@@ -3668,12 +3774,12 @@
         <v>18</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="2" t="s">
-        <v>100</v>
+        <v>112</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>6</v>
@@ -3685,12 +3791,12 @@
         <v>11</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="2" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>92</v>
@@ -3702,12 +3808,12 @@
         <v>35</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="2" t="s">
-        <v>123</v>
+        <v>135</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>29</v>
@@ -3719,12 +3825,12 @@
         <v>11</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="2" t="s">
-        <v>124</v>
+        <v>136</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>26</v>
@@ -3736,7 +3842,7 @@
         <v>11</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -3753,7 +3859,7 @@
         <v>11</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>122</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>